<commit_message>
parameters have no spaces
</commit_message>
<xml_diff>
--- a/inst/extdata/ASRparameterMapping.xlsx
+++ b/inst/extdata/ASRparameterMapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\AquaSensR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F83653-AB99-41BF-8AEC-4B4FA9CA3FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572ECFAD-1476-47B0-9A83-A482E40A931E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32460" yWindow="825" windowWidth="18270" windowHeight="14325" xr2:uid="{178F5C9C-564C-4FDF-AA7C-E06704DA2294}"/>
+    <workbookView xWindow="456" yWindow="168" windowWidth="21600" windowHeight="11232" xr2:uid="{178F5C9C-564C-4FDF-AA7C-E06704DA2294}"/>
   </bookViews>
   <sheets>
     <sheet name="Continuous Parameters" sheetId="2" r:id="rId1"/>
@@ -346,18 +346,6 @@
     <t>Water Temp (F)</t>
   </si>
   <si>
-    <t>Air Temp_C</t>
-  </si>
-  <si>
-    <t>Air Temp_F</t>
-  </si>
-  <si>
-    <t>Air BP_psi</t>
-  </si>
-  <si>
-    <t>Air BP_mmHg</t>
-  </si>
-  <si>
     <t>Chlorophylla_ug_l</t>
   </si>
   <si>
@@ -379,9 +367,6 @@
     <t>Salinity_ppt</t>
   </si>
   <si>
-    <t>Sp Conductance_uS_cm</t>
-  </si>
-  <si>
     <t>Cyanobacteria_ug_l</t>
   </si>
   <si>
@@ -406,12 +391,6 @@
     <t>FDOM_mg_l</t>
   </si>
   <si>
-    <t>E. coli_#_100ml</t>
-  </si>
-  <si>
-    <t>E. coli_CFU_100ml</t>
-  </si>
-  <si>
     <t>Discharge_cfs</t>
   </si>
   <si>
@@ -433,24 +412,6 @@
     <t>Turbidity_FNU</t>
   </si>
   <si>
-    <t>Gage Height_ft</t>
-  </si>
-  <si>
-    <t>Sensor Depth_ft</t>
-  </si>
-  <si>
-    <t>Water Pressure_psi</t>
-  </si>
-  <si>
-    <t>Water Pressure_mmHg</t>
-  </si>
-  <si>
-    <t>Water Temp_C</t>
-  </si>
-  <si>
-    <t>Water Temp_F</t>
-  </si>
-  <si>
     <t>Solids</t>
   </si>
   <si>
@@ -470,6 +431,45 @@
   </si>
   <si>
     <t>Total dissolved solids</t>
+  </si>
+  <si>
+    <t>Air_Temp_C</t>
+  </si>
+  <si>
+    <t>Air_Temp_F</t>
+  </si>
+  <si>
+    <t>Air_BP_psi</t>
+  </si>
+  <si>
+    <t>Air_BP_mmHg</t>
+  </si>
+  <si>
+    <t>Sp_Conductance_uS_cm</t>
+  </si>
+  <si>
+    <t>E_coli_#_100ml</t>
+  </si>
+  <si>
+    <t>E_coli_CFU_100ml</t>
+  </si>
+  <si>
+    <t>Gage_Height_ft</t>
+  </si>
+  <si>
+    <t>Sensor_Depth_ft</t>
+  </si>
+  <si>
+    <t>Water_Pressure_psi</t>
+  </si>
+  <si>
+    <t>Water_Pressure_mmHg</t>
+  </si>
+  <si>
+    <t>Water_Temp_C</t>
+  </si>
+  <si>
+    <t>Water_Temp_F</t>
   </si>
 </sst>
 </file>
@@ -868,7 +868,7 @@
         <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="C2" t="s">
         <v>31</v>
@@ -888,7 +888,7 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="C3" t="s">
         <v>32</v>
@@ -908,7 +908,7 @@
         <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
         <v>46</v>
@@ -928,7 +928,7 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="C5" t="s">
         <v>54</v>
@@ -948,7 +948,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C6" t="s">
         <v>41</v>
@@ -968,7 +968,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
         <v>42</v>
@@ -988,7 +988,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
         <v>41</v>
@@ -1008,7 +1008,7 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
         <v>42</v>
@@ -1028,7 +1028,7 @@
         <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
         <v>57</v>
@@ -1048,7 +1048,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1068,7 +1068,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
         <v>47</v>
@@ -1088,7 +1088,7 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="C13" t="s">
         <v>36</v>
@@ -1108,7 +1108,7 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
@@ -1128,7 +1128,7 @@
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
         <v>41</v>
@@ -1148,7 +1148,7 @@
         <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
         <v>41</v>
@@ -1168,7 +1168,7 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C17" t="s">
         <v>37</v>
@@ -1188,7 +1188,7 @@
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C18" t="s">
         <v>37</v>
@@ -1208,7 +1208,7 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C19" t="s">
         <v>22</v>
@@ -1228,7 +1228,7 @@
         <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C20" t="s">
         <v>37</v>
@@ -1248,7 +1248,7 @@
         <v>44</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C21" t="s">
         <v>37</v>
@@ -1268,7 +1268,7 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="C22" t="s">
         <v>45</v>
@@ -1288,7 +1288,7 @@
         <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="C23" t="s">
         <v>59</v>
@@ -1308,7 +1308,7 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C24" t="s">
         <v>35</v>
@@ -1328,7 +1328,7 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s">
         <v>41</v>
@@ -1348,13 +1348,13 @@
         <v>43</v>
       </c>
       <c r="B26" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C26" t="s">
         <v>49</v>
       </c>
       <c r="D26" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="E26" t="s">
         <v>48</v>
@@ -1368,7 +1368,7 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C27" t="s">
         <v>38</v>
@@ -1385,19 +1385,19 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="B28" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="C28" t="s">
         <v>37</v>
       </c>
       <c r="D28" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="E28" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="F28" t="s">
         <v>37</v>
@@ -1405,19 +1405,19 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="B29" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="C29" t="s">
         <v>37</v>
       </c>
       <c r="D29" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="E29" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
         <v>37</v>
@@ -1428,7 +1428,7 @@
         <v>8</v>
       </c>
       <c r="B30" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C30" t="s">
         <v>40</v>
@@ -1448,7 +1448,7 @@
         <v>8</v>
       </c>
       <c r="B31" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C31" t="s">
         <v>55</v>
@@ -1468,7 +1468,7 @@
         <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C32" t="s">
         <v>34</v>
@@ -1488,7 +1488,7 @@
         <v>24</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="C33" t="s">
         <v>34</v>
@@ -1508,7 +1508,7 @@
         <v>24</v>
       </c>
       <c r="B34" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C34" t="s">
         <v>46</v>
@@ -1528,7 +1528,7 @@
         <v>24</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C35" t="s">
         <v>54</v>
@@ -1548,7 +1548,7 @@
         <v>0</v>
       </c>
       <c r="B36" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C36" t="s">
         <v>31</v>
@@ -1568,7 +1568,7 @@
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C37" t="s">
         <v>32</v>

</xml_diff>